<commit_message>
docs(custos): sem o chip do WhatsApp na implantacao e sem o projeto nas fontes
Planilha: sai a linha do chip pre-pago (implantacao passa a R$ 76) e a linha do proprio projeto
na aba Fontes. CUSTOS-OPERACIONAIS.md e documentos do TCC e tecnico acompanham.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tcc/ShivaZen-Custos-Operacionais.xlsx
+++ b/docs/tcc/ShivaZen-Custos-Operacionais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafae\Documents\shivazen-app\docs\tcc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A4A13DD-87C8-4FC7-AF4F-766AF0DE3F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F5393C-389C-4A73-89C5-EF8B2075E267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="125">
   <si>
     <t>Custo do sistema: clínica com até 60 atendimentos por mês</t>
   </si>
@@ -216,15 +216,6 @@
     <t>Nos anos seguintes entra no custo mensal</t>
   </si>
   <si>
-    <t>Chip pré-pago para o número do WhatsApp</t>
-  </si>
-  <si>
-    <t>Operadora</t>
-  </si>
-  <si>
-    <t>Estimativa. O número não pode estar em uso no aplicativo WhatsApp comum</t>
-  </si>
-  <si>
     <t>Primeiro crédito de SMS</t>
   </si>
   <si>
@@ -418,15 +409,6 @@
   </si>
   <si>
     <t>https://www.bcb.gov.br/estabilidadefinanceira/historicocotacoes</t>
-  </si>
-  <si>
-    <t>Premissas e estimativa de consumo</t>
-  </si>
-  <si>
-    <t>Projeto</t>
-  </si>
-  <si>
-    <t>docs/CUSTOS-OPERACIONAIS.md</t>
   </si>
 </sst>
 </file>
@@ -496,7 +478,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -511,11 +493,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF1EFE8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -546,7 +523,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -604,9 +581,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -925,7 +899,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.140625" customWidth="1"/>
@@ -952,12 +926,12 @@
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
@@ -966,12 +940,12 @@
       <c r="B5" s="5">
         <v>60</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
@@ -980,12 +954,12 @@
       <c r="B6" s="6">
         <v>1</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
@@ -994,12 +968,12 @@
       <c r="B7" s="6">
         <v>1.25</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
@@ -1008,12 +982,12 @@
       <c r="B8" s="7">
         <v>5.0999999999999996</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
@@ -1022,12 +996,12 @@
       <c r="B9" s="8">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
@@ -1037,12 +1011,12 @@
         <f>B8*(1+B9)</f>
         <v>5.2784999999999993</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
@@ -1051,12 +1025,12 @@
       <c r="B11" s="10">
         <v>5</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
@@ -1065,12 +1039,12 @@
       <c r="B12" s="10">
         <v>7</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="31"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
@@ -1079,12 +1053,12 @@
       <c r="B13" s="7">
         <v>40</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
@@ -1093,12 +1067,12 @@
       <c r="B14" s="11">
         <v>0.12</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
@@ -1107,12 +1081,12 @@
       <c r="B15" s="11">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -1121,12 +1095,12 @@
       <c r="B16" s="7">
         <v>100</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
     </row>
     <row r="18" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
@@ -1369,148 +1343,127 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
         <v>60</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="13">
-        <v>1</v>
-      </c>
-      <c r="D31" s="27">
-        <v>20</v>
+      <c r="C31" s="27">
+        <v>300</v>
+      </c>
+      <c r="D31" s="15">
+        <f>B14</f>
+        <v>0.12</v>
       </c>
       <c r="E31" s="14">
         <f>C31*D31</f>
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>63</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="28">
-        <v>300</v>
-      </c>
-      <c r="D32" s="15">
-        <f>B14</f>
-        <v>0.12</v>
+      <c r="C32" s="13">
+        <v>1</v>
+      </c>
+      <c r="D32" s="16">
+        <v>0</v>
       </c>
       <c r="E32" s="14">
         <f>C32*D32</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="20">
+        <f>SUM(E30:E32)</f>
+        <v>76</v>
+      </c>
+      <c r="F33" s="18"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="25"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+    </row>
+    <row r="35" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C33" s="13">
-        <v>1</v>
-      </c>
-      <c r="D33" s="16">
-        <v>0</v>
-      </c>
-      <c r="E33" s="14">
-        <f>C33*D33</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="12" t="s">
+      <c r="B35" s="26" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="17" t="s">
+      <c r="C35" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="20">
-        <f>SUM(E30:E33)</f>
-        <v>96</v>
-      </c>
-      <c r="F34" s="18"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="25"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
+      <c r="D35" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="E35" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" s="26" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="36" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="C36" s="26" t="s">
+      <c r="A36" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="26" t="s">
+      <c r="B36" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="C36" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="F36" s="26" t="s">
-        <v>4</v>
+      <c r="D36" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E36" s="24">
+        <f>B16-E21</f>
+        <v>92.8</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="E37" s="24">
-        <f>B16-E21</f>
-        <v>92.8</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="E37" s="28"/>
       <c r="F37" s="12" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
         <v>80</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="E38" s="29"/>
-      <c r="F38" s="12" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1535,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.7109375" customWidth="1"/>
@@ -1546,231 +1499,217 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>